<commit_message>
Feat: Adding programme filtering to the semantic searches
</commit_message>
<xml_diff>
--- a/exchange_students.xlsx
+++ b/exchange_students.xlsx
@@ -651,22 +651,22 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2025-12-31; 2026-08-16</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-07-30; 2026-12-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2025-12-01; 2026-07-31</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-06-14; 2026-09-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -966,22 +966,22 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2027-03-13; 2027-03-13</t>
+          <t>2027-03-13</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-11-30; 2026-11-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1071,22 +1071,22 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-08-31; 2026-09-02</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-10-24; 2026-10-24</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-09-13; 2026-09-13</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1176,22 +1176,22 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2027-05-08; 2027-05-08</t>
+          <t>2027-05-08</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>2026-11-30; 2026-11-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1281,22 +1281,22 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-08-31; 2026-08-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-10-24; 2026-10-24</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-09-13; 2026-09-13</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1386,22 +1386,22 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-25; 2026-10-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-12-30; 2026-12-30</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-11-01; 2026-11-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1487,22 +1487,22 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-08-30; 2026-08-30</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2026-10-24; 2026-10-24</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-09-13; 2026-09-13</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1592,22 +1592,22 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2027-03-13; 2027-03-13</t>
+          <t>2027-03-13</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>2026-11-30; 2026-11-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1693,22 +1693,22 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-05-03; 2026-07-31</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2026-07-30; 2026-10-24</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>2026-02-15; 2026-07-01</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-06-30; 2026-07-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1794,22 +1794,22 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-08-30; 2026-09-06</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-10-24; 2026-10-24</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-08-30; 2026-08-30</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -1899,22 +1899,22 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-05-17; 2026-12-31; 2026-12-31</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2026-08-17; 2027-03-13; 2027-03-13</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>2026-04-17; 2026-12-01; 2026-12-01</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-05-30; 2026-12-31; 2026-12-31</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2089,22 +2089,22 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-10-25; 2026-10-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2026-12-30; 2026-12-30</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>2026-09-25; 2026-09-25</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-10-25; 2026-10-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2299,22 +2299,22 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-08-16</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2026-07-30; 2026-12-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-07-31</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-09-13</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2517,22 +2517,22 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2025-07-31; 2025-07-31; 2026-07-31; 2026-07-31; 2026-12-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2026-07-30; 2026-07-30; 2027-07-30; 2027-07-30; 2027-03-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>2025-07-01; 2025-07-31; 2026-07-31; 2026-07-31; 2026-12-01</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31; 2027-07-31; 2026-07-31; 2026-12-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -2832,22 +2832,22 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2026-05-31; 2026-12-31</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-12-30; 2027-05-08</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2026-05-01; 2026-12-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>2026-11-15; 2027-01-10</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -3886,22 +3886,22 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>2026-10-25; 2026-10-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2026-12-30; 2026-12-30</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>2026-11-01; 2026-11-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="T33" t="inlineStr"/>
@@ -3983,22 +3983,22 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4084,22 +4084,22 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4613,22 +4613,22 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-05-03; 2026-07-31; 2026-07-31; 2027-03-14</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>2026-07-30; 2026-07-30; 2027-05-08; 2027-07-30; 2027-05-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-02-15; 2026-07-31; 2026-06-30; 2026-11-30</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-06-30; 2027-05-09; 2026-07-01; 2027-03-21</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="T40" t="inlineStr"/>
@@ -4823,22 +4823,22 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>2026-10-25; 2027-03-14</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>2026-12-30; 2027-05-08</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-11-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>2026-11-08; 2027-03-21</t>
+          <t>2026-11-08</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
@@ -4928,22 +4928,22 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-05-03; 2026-07-31; 2026-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>2026-07-30; 2026-07-30; 2026-12-30; 2027-05-08; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-02-15; 2026-07-31; 2026-07-31; 2026-06-30</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-06-30; 2026-09-13; 2027-05-09; 2026-07-01</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
@@ -5348,22 +5348,22 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31; 2026-10-25; 2026-10-25</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-05-08; 2026-12-30; 2026-12-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-05-31; 2026-07-31; 2026-05-31</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-06-01; 2026-11-08; 2026-06-01</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
@@ -5768,22 +5768,22 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-03-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>2026-12-30; 2027-05-08</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-11-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>2026-09-13; 2027-03-21</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5881,22 +5881,22 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>2027-05-08; 2027-05-08</t>
+          <t>2027-05-08</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>2027-02-12; 2027-02-12</t>
+          <t>2027-02-12</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
@@ -5986,22 +5986,22 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>2026-08-30; 2026-08-30</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>2026-10-24; 2026-10-24</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>2026-08-09; 2026-08-09</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>2026-09-06; 2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6091,22 +6091,22 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>2026-10-25; 2026-10-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>2026-12-30; 2026-12-30</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>2026-09-25; 2026-09-25</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>2026-10-25; 2026-10-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="T54" t="inlineStr"/>
@@ -6196,22 +6196,22 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>2027-03-13; 2027-03-13</t>
+          <t>2027-03-13</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>2026-12-01; 2026-12-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="T55" t="inlineStr"/>
@@ -6301,22 +6301,22 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>2027-05-08; 2027-05-08</t>
+          <t>2027-05-08</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>2027-02-12; 2027-02-12</t>
+          <t>2027-02-12</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="T56" t="inlineStr"/>
@@ -6406,22 +6406,22 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>2026-05-10; 2026-12-31; 2026-12-31</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>2026-08-15; 2027-05-08; 2027-05-08</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>2026-04-10; 2026-12-01; 2026-12-01</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>2026-05-09; 2026-12-31; 2026-12-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="T57" t="inlineStr"/>
@@ -6515,22 +6515,22 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>2027-03-13; 2027-03-13</t>
+          <t>2027-03-13</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>2026-12-01; 2026-12-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="T58" t="inlineStr"/>
@@ -6620,22 +6620,22 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-03-14; 2027-03-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>2027-02-25; 2027-05-08; 2027-05-08</t>
+          <t>2027-02-25</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>2026-04-10; 2027-02-12; 2027-02-12</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>2026-05-10; 2027-03-14; 2027-03-14</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="T59" t="inlineStr"/>
@@ -6725,22 +6725,22 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>2026-08-30; 2026-08-30</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>2026-10-24; 2026-10-24</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>2026-08-30; 2026-08-30</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
@@ -6830,22 +6830,22 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>2026-08-30; 2026-10-25</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>2026-12-30; 2026-12-30</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-09-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>2026-08-30; 2026-10-25</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
@@ -6939,22 +6939,22 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>2027-05-08; 2027-05-08</t>
+          <t>2027-05-08</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>2027-02-12; 2027-02-12</t>
+          <t>2027-02-12</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="T62" t="inlineStr"/>
@@ -7149,22 +7149,22 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>2026-08-30; 2027-03-14</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>2026-10-31; 2027-05-08</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-02-12</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>2026-08-30; 2027-03-14</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="T64" t="inlineStr"/>
@@ -7254,22 +7254,22 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>2027-05-07; 2027-05-08</t>
+          <t>2027-05-07</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>2027-02-12; 2027-02-12</t>
+          <t>2027-02-12</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="T65" t="inlineStr"/>
@@ -8308,22 +8308,22 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>2026-08-16; 2026-09-30; 2027-03-14</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>2026-10-24; 2027-06-14; 2027-05-08</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>2026-07-07; 2026-08-31; 2027-02-12</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>2026-09-13; 2026-08-31; 2027-03-14</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -9568,22 +9568,22 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-10-25</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>2026-07-30; 2026-12-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-09-25</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>2026-06-30; 2026-10-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="T87" t="inlineStr"/>
@@ -11260,22 +11260,22 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11377,22 +11377,22 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-07-31</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11494,22 +11494,22 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>2025-06-30; 2026-07-01</t>
+          <t>2025-06-30</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11611,22 +11611,22 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-07-31</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -13109,22 +13109,22 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>2026-05-03; 2026-07-31; 2026-12-31</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-05-08; 2027-03-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>2026-02-15; 2026-07-31; 2026-11-30</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>2026-06-30; 2027-05-09; 2027-01-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="T120" t="inlineStr"/>
@@ -13315,22 +13315,22 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-05-03; 2026-07-31; 2026-07-31; 2026-10-25</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>2026-07-30; 2026-07-30; 2027-05-08; 2027-07-30; 2026-12-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-02-15; 2026-07-31; 2026-06-30; 2026-07-31</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-06-30; 2027-05-09; 2026-07-01; 2026-11-08</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="T122" t="inlineStr"/>
@@ -13638,22 +13638,22 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>2026-12-30; 2027-05-08</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>2026-08-30; 2027-05-09</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
@@ -13755,22 +13755,22 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>2027-05-08; 2027-05-08</t>
+          <t>2027-05-08</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>2026-11-30; 2027-02-12</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>2027-03-21; 2027-02-13</t>
+          <t>2027-03-21</t>
         </is>
       </c>
       <c r="T126" t="inlineStr"/>
@@ -14074,22 +14074,22 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>2027-03-13; 2027-03-13</t>
+          <t>2027-03-13</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>2026-11-30; 2026-12-01</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>2027-01-03; 2026-12-02</t>
+          <t>2027-01-03</t>
         </is>
       </c>
       <c r="T129" t="inlineStr"/>
@@ -14817,22 +14817,22 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>2027-03-14; 2027-03-14</t>
+          <t>2027-03-14</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>2027-05-08; 2027-05-08</t>
+          <t>2027-05-08</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>2026-11-30; 2027-02-12</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>2027-03-21; 2027-02-13</t>
+          <t>2027-03-21</t>
         </is>
       </c>
       <c r="T136" t="inlineStr"/>
@@ -14922,22 +14922,22 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-07-31; 2027-03-14; 2027-03-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>2026-10-24; 2026-10-24; 2027-05-08; 2027-05-08</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-05-31; 2026-11-30; 2027-02-12</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S137" t="inlineStr">
         <is>
-          <t>2026-09-13; 2026-06-01; 2027-03-21; 2027-02-13</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="T137" t="inlineStr">
@@ -15455,22 +15455,22 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>2026-12-31; 2026-12-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>2027-05-08; 2027-05-08</t>
+          <t>2027-05-08</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
         <is>
-          <t>2026-11-30; 2026-12-01</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="S142" t="inlineStr">
         <is>
-          <t>2027-01-03; 2026-12-02</t>
+          <t>2027-01-03</t>
         </is>
       </c>
       <c r="T142" t="inlineStr"/>
@@ -15564,22 +15564,22 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>2026-10-25; 2026-10-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>2026-12-30; 2026-12-30</t>
+          <t>2026-12-30</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>2026-07-31; 2026-09-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="S143" t="inlineStr">
         <is>
-          <t>2026-11-08; 2026-09-26</t>
+          <t>2026-11-08</t>
         </is>
       </c>
       <c r="T143" t="inlineStr"/>
@@ -16089,22 +16089,22 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>2026-05-03; 2027-03-14</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-05-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
         <is>
-          <t>2026-02-15; 2026-11-30</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="S148" t="inlineStr">
         <is>
-          <t>2026-06-30; 2027-03-21</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="T148" t="inlineStr"/>
@@ -16190,22 +16190,22 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>2026-05-03; 2026-12-31</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-03-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
         <is>
-          <t>2026-02-15; 2026-11-30</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="S149" t="inlineStr">
         <is>
-          <t>2026-06-30; 2027-01-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="T149" t="inlineStr"/>
@@ -16485,22 +16485,22 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="S152" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T152" t="inlineStr">
@@ -16594,22 +16594,22 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="S153" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T153" t="inlineStr">
@@ -16703,22 +16703,22 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="S154" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T154" t="inlineStr">
@@ -16820,22 +16820,22 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="S155" t="inlineStr">
         <is>
-          <t>2026-07-31; 2027-07-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="T155" t="inlineStr">
@@ -18379,22 +18379,22 @@
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>2026-07-30; 2027-07-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
         <is>
-          <t>2025-07-01; 2026-07-01</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="S170" t="inlineStr">
         <is>
-          <t>2025-07-31; 2026-07-31</t>
+          <t>2025-07-31</t>
         </is>
       </c>
       <c r="T170" t="inlineStr">

</xml_diff>